<commit_message>
Add new feature: version 4
</commit_message>
<xml_diff>
--- a/data/UNSPED_Karbon_Veri_Girisi_v3_updated (4).xlsx
+++ b/data/UNSPED_Karbon_Veri_Girisi_v3_updated (4).xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="12" activeTab="19" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1.1_Stationary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="1.2_Mobile" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="1.4_Refrigerants" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="2.1_Electricity" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="3.1_Freight" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="3.2_ProductShipment" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="3.3_Commuting" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="3.4_BusinessTravel" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="3.5_FlightsHotels" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="4.1_Purchased" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="4.2_Capital" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="4.3_Waste" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="4.4_LeasedEquipment" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="4.5_Services" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="6.1_TDLosses" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="PERSONNEL" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="TOTAL_EMISSIONS" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="IMPACT_ANALYSIS" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="PER_CAPITA" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.1_Stationary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.2_Mobile" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.4_Refrigerants" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.1_Electricity" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.1_Freight" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.2_ProductShipment" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.3_Commuting" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.4_BusinessTravel" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.5_FlightsHotels" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.1_Purchased" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.2_Capital" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.3_Waste" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.4_LeasedEquipment" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.5_Services" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6.1_TDLosses" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERSONNEL" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTAL_EMISSIONS" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMPACT_ANALYSIS" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PER_CAPITA" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>